<commit_message>
fix 3, sudah stop + no dobel excel. penambahan fitur menu belum rename
</commit_message>
<xml_diff>
--- a/uploads/data_entry.xlsx
+++ b/uploads/data_entry.xlsx
@@ -222,10 +222,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -543,7 +543,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -622,14 +622,14 @@
       <c r="G2" s="11">
         <v>153600</v>
       </c>
-      <c r="H2" s="8">
+      <c r="H2" s="7">
         <v>46084</v>
       </c>
       <c r="I2" s="5"/>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="8" t="s">
         <v>1</v>
       </c>
     </row>
@@ -643,10 +643,10 @@
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
       <c r="G3" s="11"/>
-      <c r="H3" s="8"/>
+      <c r="H3" s="7"/>
       <c r="I3" s="5"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
@@ -670,14 +670,14 @@
       <c r="G4" s="11">
         <v>235800</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <v>46084</v>
       </c>
       <c r="I4" s="5"/>
-      <c r="J4" s="7" t="s">
+      <c r="J4" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="8" t="s">
         <v>45</v>
       </c>
     </row>
@@ -691,10 +691,10 @@
       <c r="E5" s="10"/>
       <c r="F5" s="10"/>
       <c r="G5" s="11"/>
-      <c r="H5" s="8"/>
+      <c r="H5" s="7"/>
       <c r="I5" s="5"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
     </row>
     <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
@@ -718,14 +718,14 @@
       <c r="G6" s="11">
         <v>168500</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>46084</v>
       </c>
       <c r="I6" s="5"/>
-      <c r="J6" s="7" t="s">
+      <c r="J6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="8" t="s">
         <v>47</v>
       </c>
     </row>
@@ -739,10 +739,10 @@
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="8"/>
+      <c r="H7" s="7"/>
       <c r="I7" s="5"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
@@ -766,14 +766,14 @@
       <c r="G8" s="11">
         <v>234100</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="7">
         <v>46084</v>
       </c>
       <c r="I8" s="5"/>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="K8" s="8" t="s">
         <v>1</v>
       </c>
     </row>
@@ -787,10 +787,10 @@
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
       <c r="G9" s="11"/>
-      <c r="H9" s="8"/>
+      <c r="H9" s="7"/>
       <c r="I9" s="5"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
     </row>
     <row r="10" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
@@ -814,14 +814,14 @@
       <c r="G10" s="11">
         <v>240700</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="7">
         <v>46084</v>
       </c>
       <c r="I10" s="5"/>
-      <c r="J10" s="7" t="s">
+      <c r="J10" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="K10" s="8" t="s">
         <v>45</v>
       </c>
     </row>
@@ -835,10 +835,10 @@
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
       <c r="G11" s="11"/>
-      <c r="H11" s="8"/>
+      <c r="H11" s="7"/>
       <c r="I11" s="5"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
     </row>
     <row r="12" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
@@ -862,14 +862,14 @@
       <c r="G12" s="11">
         <v>210900</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="7">
         <v>46084</v>
       </c>
       <c r="I12" s="5"/>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="K12" s="8" t="s">
         <v>47</v>
       </c>
     </row>
@@ -883,10 +883,10 @@
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
       <c r="G13" s="11"/>
-      <c r="H13" s="8"/>
+      <c r="H13" s="7"/>
       <c r="I13" s="5"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
     </row>
     <row r="14" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
@@ -910,14 +910,14 @@
       <c r="G14" s="11">
         <v>168500</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="7">
         <v>46084</v>
       </c>
       <c r="I14" s="5"/>
-      <c r="J14" s="7" t="s">
+      <c r="J14" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="8" t="s">
         <v>1</v>
       </c>
     </row>
@@ -931,10 +931,10 @@
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="11"/>
-      <c r="H15" s="8"/>
+      <c r="H15" s="7"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
     </row>
     <row r="16" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
@@ -958,14 +958,14 @@
       <c r="G16" s="11">
         <v>196800</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="7">
         <v>46084</v>
       </c>
       <c r="I16" s="5"/>
-      <c r="J16" s="7" t="s">
+      <c r="J16" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="K16" s="8" t="s">
         <v>45</v>
       </c>
     </row>
@@ -979,10 +979,10 @@
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
       <c r="G17" s="11"/>
-      <c r="H17" s="8"/>
+      <c r="H17" s="7"/>
       <c r="I17" s="5"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="J25" s="4" t="s">
@@ -991,6 +991,62 @@
     </row>
   </sheetData>
   <mergeCells count="72">
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:G7"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="A4:A5"/>
@@ -1007,62 +1063,6 @@
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="K10:K11"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="K12:K13"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="K16:K17"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="J12:J13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>